<commit_message>
Refine OrganizationCode rule and AreaMgmt alignment
</commit_message>
<xml_diff>
--- a/templates/test_files/Data Dictionary_BdCH_AreaMgmt_v0.9.4.xlsx
+++ b/templates/test_files/Data Dictionary_BdCH_AreaMgmt_v0.9.4.xlsx
@@ -9558,12 +9558,12 @@
       </c>
       <c r="B4" s="245" t="inlineStr">
         <is>
-          <t>DataDic</t>
+          <t>BdCH</t>
         </is>
       </c>
       <c r="C4" s="248" t="inlineStr">
         <is>
-          <t>REQUIRED</t>
+          <t>user defined name (small or capital letters), max 7 chars</t>
         </is>
       </c>
       <c r="D4" s="245" t="inlineStr">
@@ -9712,7 +9712,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://example.com/DataDic/data_dictionary_area_management</t>
+          <t>https://example.com/BdCH/data_dictionary_area_management</t>
         </is>
       </c>
       <c r="C11" s="248" t="inlineStr">
@@ -26036,7 +26036,7 @@
       <c r="E7" s="198" t="n"/>
       <c r="F7" s="198" t="inlineStr">
         <is>
-          <t>DataDic_AreaMgmt</t>
+          <t>BdCH_AreaMgmt</t>
         </is>
       </c>
       <c r="G7" s="198" t="inlineStr">

</xml_diff>